<commit_message>
now exeval_ppk accepted in plot fit
No need to x$metrics in function
</commit_message>
<xml_diff>
--- a/external_evaluation_results.xlsx
+++ b/external_evaluation_results.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t xml:space="preserve">OCC</t>
   </si>
@@ -68,19 +68,61 @@
     <t xml:space="preserve">Fit_Class</t>
   </si>
   <si>
+    <t xml:space="preserve">Acceptable</t>
+  </si>
+  <si>
     <t xml:space="preserve">Very Poor</t>
   </si>
   <si>
     <t xml:space="preserve">Poor</t>
   </si>
   <si>
+    <t xml:space="preserve">Excellent</t>
+  </si>
+  <si>
     <t xml:space="preserve">Parameter</t>
   </si>
   <si>
     <t xml:space="preserve">Value</t>
   </si>
   <si>
-    <t xml:space="preserve">Evaluation type</t>
+    <t xml:space="preserve">Num IDs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Num Occasion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Num of Ref Occasion</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Drug Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tacrolimus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Han_etal_2011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluation</t>
   </si>
   <si>
     <t xml:space="preserve">Progressive</t>
@@ -89,13 +131,7 @@
     <t xml:space="preserve">Assessment</t>
   </si>
   <si>
-    <t xml:space="preserve">a_priori</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mapbayr</t>
+    <t xml:space="preserve">Bayesian_forecasting</t>
   </si>
 </sst>
 </file>
@@ -452,28 +488,54 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>-22.3549563482925</v>
+        <v>14.5000610167097</v>
       </c>
       <c r="C2" t="n">
-        <v>-40.1561765410529</v>
+        <v>-7.96369857287708</v>
       </c>
       <c r="D2" t="n">
-        <v>-4.55373615553204</v>
+        <v>36.9638206062964</v>
       </c>
       <c r="E2" t="n">
-        <v>31.0342045964223</v>
+        <v>31.517370501966</v>
       </c>
       <c r="F2" t="n">
-        <v>36.0660451859888</v>
+        <v>38.5464344027266</v>
       </c>
       <c r="G2" t="n">
-        <v>30.7692307692308</v>
+        <v>23.0769230769231</v>
       </c>
       <c r="H2" t="n">
-        <v>61.5384615384615</v>
+        <v>69.2307692307692</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="n">
+        <v>5.86313147165341</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-27.4579279521439</v>
+      </c>
+      <c r="D3" t="n">
+        <v>39.1841908954507</v>
+      </c>
+      <c r="E3" t="n">
+        <v>40.5227802012222</v>
+      </c>
+      <c r="F3" t="n">
+        <v>44.5765855712491</v>
+      </c>
+      <c r="G3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H3" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -518,25 +580,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>168</v>
+        <v>264</v>
       </c>
       <c r="D2" t="n">
-        <v>4.51798546657624</v>
+        <v>10.2023965957545</v>
       </c>
       <c r="E2" t="n">
-        <v>9.4</v>
+        <v>8.4</v>
       </c>
       <c r="F2" t="n">
-        <v>-51.9363248236571</v>
+        <v>21.4571023304112</v>
       </c>
       <c r="G2" t="n">
-        <v>51.9363248236571</v>
+        <v>21.4571023304112</v>
       </c>
       <c r="H2" t="n">
-        <v>0.269738183618842</v>
+        <v>0.0460407240417736</v>
       </c>
     </row>
     <row r="3">
@@ -544,25 +606,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>408</v>
+        <v>744</v>
       </c>
       <c r="D3" t="n">
-        <v>4.65174183449702</v>
+        <v>5.15771484090867</v>
       </c>
       <c r="E3" t="n">
-        <v>6.2</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>-24.9719058952093</v>
+        <v>28.9428710227167</v>
       </c>
       <c r="G3" t="n">
-        <v>24.9719058952093</v>
+        <v>28.9428710227167</v>
       </c>
       <c r="H3" t="n">
-        <v>0.062359608403919</v>
+        <v>0.0837689783037613</v>
       </c>
     </row>
     <row r="4">
@@ -570,25 +632,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>72</v>
+        <v>168</v>
       </c>
       <c r="D4" t="n">
-        <v>14.2686207675188</v>
+        <v>16.7912735362117</v>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-28.6568961624059</v>
+        <v>39.9272794684308</v>
       </c>
       <c r="G4" t="n">
-        <v>28.6568961624059</v>
+        <v>39.9272794684308</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0821217697662911</v>
+        <v>0.159418764575018</v>
       </c>
     </row>
     <row r="5">
@@ -596,25 +658,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>168</v>
+        <v>264</v>
       </c>
       <c r="D5" t="n">
-        <v>11.8718281741435</v>
+        <v>12.4741682451794</v>
       </c>
       <c r="E5" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="F5" t="n">
-        <v>-24.3832600373027</v>
+        <v>-21.049568068485</v>
       </c>
       <c r="G5" t="n">
-        <v>24.3832600373027</v>
+        <v>21.049568068485</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0594543370046724</v>
+        <v>0.0443084315869782</v>
       </c>
     </row>
     <row r="6">
@@ -622,25 +684,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="D6" t="n">
-        <v>5.34217883377462</v>
+        <v>8.26995833236441</v>
       </c>
       <c r="E6" t="n">
-        <v>6.4</v>
+        <v>12.6</v>
       </c>
       <c r="F6" t="n">
-        <v>-16.5284557222716</v>
+        <v>-34.3654100605999</v>
       </c>
       <c r="G6" t="n">
-        <v>16.5284557222716</v>
+        <v>34.3654100605999</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0273189848563092</v>
+        <v>0.118098140863318</v>
       </c>
     </row>
     <row r="7">
@@ -648,155 +710,155 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="D7" t="n">
-        <v>8.85385618643503</v>
+        <v>7.23617714992378</v>
       </c>
       <c r="E7" t="n">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="F7" t="n">
-        <v>42.8041320392746</v>
+        <v>24.7616749986858</v>
       </c>
       <c r="G7" t="n">
-        <v>42.8041320392746</v>
+        <v>24.7616749986858</v>
       </c>
       <c r="H7" t="n">
-        <v>0.183219371963566</v>
+        <v>0.0613140548740541</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>96</v>
+        <v>241</v>
       </c>
       <c r="D8" t="n">
-        <v>8.56605220650252</v>
+        <v>14.3617388330959</v>
       </c>
       <c r="E8" t="n">
-        <v>7.8</v>
+        <v>16.1</v>
       </c>
       <c r="F8" t="n">
-        <v>9.82118213464766</v>
+        <v>-10.7966532105844</v>
       </c>
       <c r="G8" t="n">
-        <v>9.82118213464766</v>
+        <v>10.7966532105844</v>
       </c>
       <c r="H8" t="n">
-        <v>0.00964556185219224</v>
+        <v>0.0116567720549622</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>72</v>
+        <v>242</v>
       </c>
       <c r="D9" t="n">
-        <v>7.020954657218</v>
+        <v>13.5704359612845</v>
       </c>
       <c r="E9" t="n">
-        <v>9.3</v>
+        <v>15.5</v>
       </c>
       <c r="F9" t="n">
-        <v>-24.5058639008817</v>
+        <v>-12.4488002497776</v>
       </c>
       <c r="G9" t="n">
-        <v>24.5058639008817</v>
+        <v>12.4488002497776</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0600537365528537</v>
+        <v>0.0154972627658864</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>96</v>
+        <v>248</v>
       </c>
       <c r="D10" t="n">
-        <v>10.0676105455754</v>
+        <v>9.30584726965556</v>
       </c>
       <c r="E10" t="n">
-        <v>9.7</v>
+        <v>7.3</v>
       </c>
       <c r="F10" t="n">
-        <v>3.78979943892144</v>
+        <v>27.4773598582954</v>
       </c>
       <c r="G10" t="n">
-        <v>3.78979943892144</v>
+        <v>27.4773598582954</v>
       </c>
       <c r="H10" t="n">
-        <v>0.00143625797872493</v>
+        <v>0.0755005304782263</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>97</v>
+        <v>192</v>
       </c>
       <c r="D11" t="n">
-        <v>13.8694497400213</v>
+        <v>8.56326391428382</v>
       </c>
       <c r="E11" t="n">
-        <v>35</v>
+        <v>12.1</v>
       </c>
       <c r="F11" t="n">
-        <v>-60.3730007427963</v>
+        <v>-29.229223848894</v>
       </c>
       <c r="G11" t="n">
-        <v>60.3730007427963</v>
+        <v>29.229223848894</v>
       </c>
       <c r="H11" t="n">
-        <v>0.364489921868968</v>
+        <v>0.0854347526808754</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>98</v>
+        <v>216</v>
       </c>
       <c r="D12" t="n">
-        <v>13.5126426537763</v>
+        <v>11.1623444729648</v>
       </c>
       <c r="E12" t="n">
-        <v>37.6</v>
+        <v>6.1</v>
       </c>
       <c r="F12" t="n">
-        <v>-64.0621206016589</v>
+        <v>82.9892536551611</v>
       </c>
       <c r="G12" t="n">
-        <v>64.0621206016589</v>
+        <v>82.9892536551611</v>
       </c>
       <c r="H12" t="n">
-        <v>0.410395529598149</v>
+        <v>0.688721622224067</v>
       </c>
     </row>
     <row r="13">
@@ -804,25 +866,25 @@
         <v>9</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="D13" t="n">
-        <v>12.7406341626605</v>
+        <v>8.15721488627148</v>
       </c>
       <c r="E13" t="n">
-        <v>20.4</v>
+        <v>4.7</v>
       </c>
       <c r="F13" t="n">
-        <v>-37.5459109673503</v>
+        <v>73.5577635376911</v>
       </c>
       <c r="G13" t="n">
-        <v>37.5459109673503</v>
+        <v>73.5577635376911</v>
       </c>
       <c r="H13" t="n">
-        <v>0.14096954303682</v>
+        <v>0.541074457666687</v>
       </c>
     </row>
     <row r="14">
@@ -830,25 +892,285 @@
         <v>10</v>
       </c>
       <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>288</v>
+      </c>
+      <c r="D14" t="n">
+        <v>9.33860580328076</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-2.72285621582539</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2.72285621582539</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.000741394597205896</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>1</v>
       </c>
-      <c r="C14" t="n">
-        <v>216</v>
-      </c>
-      <c r="D14" t="n">
-        <v>7.99187992229855</v>
-      </c>
-      <c r="E14" t="n">
-        <v>9.3</v>
-      </c>
-      <c r="F14" t="n">
-        <v>-14.0658072871123</v>
-      </c>
-      <c r="G14" t="n">
-        <v>14.0658072871123</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.0197846934638182</v>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>360</v>
+      </c>
+      <c r="D15" t="n">
+        <v>10.6950977727138</v>
+      </c>
+      <c r="E15" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>27.3225925323066</v>
+      </c>
+      <c r="G15" t="n">
+        <v>27.3225925323066</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.0746524062686456</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>37848</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4.85953650616147</v>
+      </c>
+      <c r="E16" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-50.9137726650356</v>
+      </c>
+      <c r="G16" t="n">
+        <v>50.9137726650356</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.259221224698693</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>240</v>
+      </c>
+      <c r="D17" t="n">
+        <v>14.9173372455131</v>
+      </c>
+      <c r="E17" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>34.3904256352534</v>
+      </c>
+      <c r="G17" t="n">
+        <v>34.3904256352534</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.118270137537389</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>432</v>
+      </c>
+      <c r="D18" t="n">
+        <v>12.3497797668135</v>
+      </c>
+      <c r="E18" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-43.3496340971858</v>
+      </c>
+      <c r="G18" t="n">
+        <v>43.3496340971858</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.187919077635989</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>336</v>
+      </c>
+      <c r="D19" t="n">
+        <v>9.77618621461461</v>
+      </c>
+      <c r="E19" t="n">
+        <v>7</v>
+      </c>
+      <c r="F19" t="n">
+        <v>39.6598030659229</v>
+      </c>
+      <c r="G19" t="n">
+        <v>39.6598030659229</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.157289997922779</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>336</v>
+      </c>
+      <c r="D20" t="n">
+        <v>8.15983019421711</v>
+      </c>
+      <c r="E20" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" t="n">
+        <v>-32.0014150481908</v>
+      </c>
+      <c r="G20" t="n">
+        <v>32.0014150481908</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.102409056508657</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>240</v>
+      </c>
+      <c r="D21" t="n">
+        <v>13.0020055973596</v>
+      </c>
+      <c r="E21" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-15.0195712590874</v>
+      </c>
+      <c r="G21" t="n">
+        <v>15.0195712590874</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.0225587520806804</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="n">
+        <v>312</v>
+      </c>
+      <c r="D22" t="n">
+        <v>9.78594349264044</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F22" t="n">
+        <v>41.8252680092818</v>
+      </c>
+      <c r="G22" t="n">
+        <v>41.8252680092818</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.174935304404825</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>9</v>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>336</v>
+      </c>
+      <c r="D23" t="n">
+        <v>8.4929161104726</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>88.7314691216132</v>
+      </c>
+      <c r="G23" t="n">
+        <v>88.7314691216132</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.78732736124798</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>10</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>480</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9.5180609190318</v>
+      </c>
+      <c r="E24" t="n">
+        <v>14</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-32.0138505783443</v>
+      </c>
+      <c r="G24" t="n">
+        <v>32.0138505783443</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.102488662885256</v>
       </c>
     </row>
   </sheetData>
@@ -899,28 +1221,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>168</v>
+        <v>264</v>
       </c>
       <c r="D2" t="n">
-        <v>4.51798546657624</v>
+        <v>10.2023965957545</v>
       </c>
       <c r="E2" t="n">
-        <v>9.4</v>
+        <v>8.4</v>
       </c>
       <c r="F2" t="n">
-        <v>-51.9363248236571</v>
+        <v>21.4571023304112</v>
       </c>
       <c r="G2" t="n">
-        <v>51.9363248236571</v>
+        <v>21.4571023304112</v>
       </c>
       <c r="H2" t="n">
-        <v>0.269738183618842</v>
+        <v>0.0460407240417736</v>
       </c>
       <c r="I2" t="n">
-        <v>51.9363248236571</v>
+        <v>21.4571023304112</v>
       </c>
       <c r="J2" t="s">
         <v>17</v>
@@ -928,63 +1250,63 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>168</v>
+        <v>360</v>
       </c>
       <c r="D3" t="n">
-        <v>8.85385618643503</v>
+        <v>10.6950977727138</v>
       </c>
       <c r="E3" t="n">
-        <v>6.2</v>
+        <v>8.4</v>
       </c>
       <c r="F3" t="n">
-        <v>42.8041320392746</v>
+        <v>27.3225925323066</v>
       </c>
       <c r="G3" t="n">
-        <v>42.8041320392746</v>
+        <v>27.3225925323066</v>
       </c>
       <c r="H3" t="n">
-        <v>0.183219371963566</v>
+        <v>0.0746524062686456</v>
       </c>
       <c r="I3" t="n">
-        <v>42.8041320392746</v>
+        <v>27.3225925323066</v>
       </c>
       <c r="J3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>97</v>
+        <v>744</v>
       </c>
       <c r="D4" t="n">
-        <v>13.8694497400213</v>
+        <v>5.15771484090867</v>
       </c>
       <c r="E4" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>-60.3730007427963</v>
+        <v>28.9428710227167</v>
       </c>
       <c r="G4" t="n">
-        <v>60.3730007427963</v>
+        <v>28.9428710227167</v>
       </c>
       <c r="H4" t="n">
-        <v>0.364489921868968</v>
+        <v>0.0837689783037613</v>
       </c>
       <c r="I4" t="n">
-        <v>60.3730007427963</v>
+        <v>28.9428710227167</v>
       </c>
       <c r="J4" t="s">
         <v>17</v>
@@ -992,66 +1314,642 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>98</v>
+        <v>37848</v>
       </c>
       <c r="D5" t="n">
-        <v>13.5126426537763</v>
+        <v>4.85953650616147</v>
       </c>
       <c r="E5" t="n">
-        <v>37.6</v>
+        <v>9.9</v>
       </c>
       <c r="F5" t="n">
-        <v>-64.0621206016589</v>
+        <v>-50.9137726650356</v>
       </c>
       <c r="G5" t="n">
-        <v>64.0621206016589</v>
+        <v>50.9137726650356</v>
       </c>
       <c r="H5" t="n">
-        <v>0.410395529598149</v>
+        <v>0.259221224698693</v>
       </c>
       <c r="I5" t="n">
-        <v>64.0621206016589</v>
+        <v>50.9137726650356</v>
       </c>
       <c r="J5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>168</v>
+      </c>
+      <c r="D6" t="n">
+        <v>16.7912735362117</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>39.9272794684308</v>
+      </c>
+      <c r="G6" t="n">
+        <v>39.9272794684308</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.159418764575018</v>
+      </c>
+      <c r="I6" t="n">
+        <v>39.9272794684308</v>
+      </c>
+      <c r="J6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>240</v>
+      </c>
+      <c r="D7" t="n">
+        <v>14.9173372455131</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>34.3904256352534</v>
+      </c>
+      <c r="G7" t="n">
+        <v>34.3904256352534</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.118270137537389</v>
+      </c>
+      <c r="I7" t="n">
+        <v>34.3904256352534</v>
+      </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>264</v>
+      </c>
+      <c r="D8" t="n">
+        <v>12.4741682451794</v>
+      </c>
+      <c r="E8" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-21.049568068485</v>
+      </c>
+      <c r="G8" t="n">
+        <v>21.049568068485</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.0443084315869782</v>
+      </c>
+      <c r="I8" t="n">
+        <v>21.049568068485</v>
+      </c>
+      <c r="J8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>432</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12.3497797668135</v>
+      </c>
+      <c r="E9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-43.3496340971858</v>
+      </c>
+      <c r="G9" t="n">
+        <v>43.3496340971858</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.187919077635989</v>
+      </c>
+      <c r="I9" t="n">
+        <v>43.3496340971858</v>
+      </c>
+      <c r="J9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>240</v>
+      </c>
+      <c r="D10" t="n">
+        <v>8.26995833236441</v>
+      </c>
+      <c r="E10" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-34.3654100605999</v>
+      </c>
+      <c r="G10" t="n">
+        <v>34.3654100605999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.118098140863318</v>
+      </c>
+      <c r="I10" t="n">
+        <v>34.3654100605999</v>
+      </c>
+      <c r="J10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>336</v>
+      </c>
+      <c r="D11" t="n">
+        <v>9.77618621461461</v>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="n">
+        <v>39.6598030659229</v>
+      </c>
+      <c r="G11" t="n">
+        <v>39.6598030659229</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.157289997922779</v>
+      </c>
+      <c r="I11" t="n">
+        <v>39.6598030659229</v>
+      </c>
+      <c r="J11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>240</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7.23617714992378</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>24.7616749986858</v>
+      </c>
+      <c r="G12" t="n">
+        <v>24.7616749986858</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.0613140548740541</v>
+      </c>
+      <c r="I12" t="n">
+        <v>24.7616749986858</v>
+      </c>
+      <c r="J12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>241</v>
+      </c>
+      <c r="D13" t="n">
+        <v>14.3617388330959</v>
+      </c>
+      <c r="E13" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-10.7966532105844</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10.7966532105844</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.0116567720549622</v>
+      </c>
+      <c r="I13" t="n">
+        <v>10.7966532105844</v>
+      </c>
+      <c r="J13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>242</v>
+      </c>
+      <c r="D14" t="n">
+        <v>13.5704359612845</v>
+      </c>
+      <c r="E14" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-12.4488002497776</v>
+      </c>
+      <c r="G14" t="n">
+        <v>12.4488002497776</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.0154972627658864</v>
+      </c>
+      <c r="I14" t="n">
+        <v>12.4488002497776</v>
+      </c>
+      <c r="J14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>248</v>
+      </c>
+      <c r="D15" t="n">
+        <v>9.30584726965556</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>27.4773598582954</v>
+      </c>
+      <c r="G15" t="n">
+        <v>27.4773598582954</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.0755005304782263</v>
+      </c>
+      <c r="I15" t="n">
+        <v>27.4773598582954</v>
+      </c>
+      <c r="J15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>336</v>
+      </c>
+      <c r="D16" t="n">
+        <v>8.15983019421711</v>
+      </c>
+      <c r="E16" t="n">
+        <v>12</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-32.0014150481908</v>
+      </c>
+      <c r="G16" t="n">
+        <v>32.0014150481908</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.102409056508657</v>
+      </c>
+      <c r="I16" t="n">
+        <v>32.0014150481908</v>
+      </c>
+      <c r="J16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>192</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8.56326391428382</v>
+      </c>
+      <c r="E17" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-29.229223848894</v>
+      </c>
+      <c r="G17" t="n">
+        <v>29.229223848894</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.0854347526808754</v>
+      </c>
+      <c r="I17" t="n">
+        <v>29.229223848894</v>
+      </c>
+      <c r="J17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>240</v>
+      </c>
+      <c r="D18" t="n">
+        <v>13.0020055973596</v>
+      </c>
+      <c r="E18" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-15.0195712590874</v>
+      </c>
+      <c r="G18" t="n">
+        <v>15.0195712590874</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.0225587520806804</v>
+      </c>
+      <c r="I18" t="n">
+        <v>15.0195712590874</v>
+      </c>
+      <c r="J18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>216</v>
+      </c>
+      <c r="D19" t="n">
+        <v>11.1623444729648</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>82.9892536551611</v>
+      </c>
+      <c r="G19" t="n">
+        <v>82.9892536551611</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.688721622224067</v>
+      </c>
+      <c r="I19" t="n">
+        <v>82.9892536551611</v>
+      </c>
+      <c r="J19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>312</v>
+      </c>
+      <c r="D20" t="n">
+        <v>9.78594349264044</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F20" t="n">
+        <v>41.8252680092818</v>
+      </c>
+      <c r="G20" t="n">
+        <v>41.8252680092818</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.174935304404825</v>
+      </c>
+      <c r="I20" t="n">
+        <v>41.8252680092818</v>
+      </c>
+      <c r="J20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
         <v>9</v>
       </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" t="n">
-        <v>12.7406341626605</v>
-      </c>
-      <c r="E6" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-37.5459109673503</v>
-      </c>
-      <c r="G6" t="n">
-        <v>37.5459109673503</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.14096954303682</v>
-      </c>
-      <c r="I6" t="n">
-        <v>37.5459109673503</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>120</v>
+      </c>
+      <c r="D21" t="n">
+        <v>8.15721488627148</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>73.5577635376911</v>
+      </c>
+      <c r="G21" t="n">
+        <v>73.5577635376911</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.541074457666687</v>
+      </c>
+      <c r="I21" t="n">
+        <v>73.5577635376911</v>
+      </c>
+      <c r="J21" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>9</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="n">
+        <v>336</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8.4929161104726</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F22" t="n">
+        <v>88.7314691216132</v>
+      </c>
+      <c r="G22" t="n">
+        <v>88.7314691216132</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.78732736124798</v>
+      </c>
+      <c r="I22" t="n">
+        <v>88.7314691216132</v>
+      </c>
+      <c r="J22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>10</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>288</v>
+      </c>
+      <c r="D23" t="n">
+        <v>9.33860580328076</v>
+      </c>
+      <c r="E23" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F23" t="n">
+        <v>-2.72285621582539</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2.72285621582539</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.000741394597205896</v>
+      </c>
+      <c r="I23" t="n">
+        <v>2.72285621582539</v>
+      </c>
+      <c r="J23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>10</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>480</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9.5180609190318</v>
+      </c>
+      <c r="E24" t="n">
+        <v>14</v>
+      </c>
+      <c r="F24" t="n">
+        <v>-32.0138505783443</v>
+      </c>
+      <c r="G24" t="n">
+        <v>32.0138505783443</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.102488662885256</v>
+      </c>
+      <c r="I24" t="n">
+        <v>32.0138505783443</v>
+      </c>
+      <c r="J24" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1067,34 +1965,74 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>